<commit_message>
Michael Nabil (LLMs EDA Bench, Adding more details
</commit_message>
<xml_diff>
--- a/LLMs Group/michael_nabil/LLMs_benchmarks_papers/LLMs_benchmarks_for_EDA_and_data_analysis.xlsx
+++ b/LLMs Group/michael_nabil/LLMs_benchmarks_papers/LLMs_benchmarks_for_EDA_and_data_analysis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="57">
   <si>
     <t xml:space="preserve">Paper Title</t>
   </si>
@@ -163,6 +163,9 @@
 3) Final Score (uses a specific formula mentioned in the paper)</t>
   </si>
   <si>
+    <t xml:space="preserve">It might be the best benchmark in terms of the variety of the used evaluation metrics, measuring different aspects of the performance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">MLAgentBench: evaluating language agents on machine learning experimentation
 </t>
   </si>
@@ -177,37 +180,9 @@
 https://dl.acm.org/doi/10.5555/3692070.3692884</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">It evaluates LLM agents on entire ML research workflows, 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">- We can tune the idea into “llms as EDA researchers“,  that can suggest analysis pipelines for different types of chaotic data.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">The paper evaluates LLM agents not just on data analysis, but also model selection, training, hparam tuning, and result understanding. It tests whether LLMs can act as autonomous ML researchers.</t>
-    </r>
+    <t xml:space="preserve">It evaluates LLM agents on entire ML research workflows. (Not specific to EDA)
+- We can tune the idea into “llms as EDA researchers“,  that can suggest analysis pipelines for different types of chaotic data.
+The paper evaluates LLM agents not just on data analysis, but also model selection, training, hparam tuning, and result understanding. It tests whether LLMs can act as autonomous ML researchers.</t>
   </si>
   <si>
     <r>
@@ -216,6 +191,7 @@
         <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1) </t>
     </r>
@@ -226,6 +202,7 @@
         <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Competence in accomplishing the objectives</t>
     </r>
@@ -235,6 +212,7 @@
         <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">: run the evaluator to obtain a single performance metric based on the final snapshot of the working directory. Then we define success as whether the performance metric is improved over baseline by 10%. then compute aggregated metrics over the performance metric of multiple runs.
 2) </t>
@@ -246,6 +224,7 @@
         <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Efficiency</t>
     </r>
@@ -255,11 +234,15 @@
         <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">: evaluating efficiency in terms of the total amount of time spent and the total number of input and output tokens consumed by the agent.</t>
     </r>
   </si>
   <si>
+    <t xml:space="preserve">The eval metrics used will not be suitable for the EDA eval, as it evaluates the performance based on the accuracy or the metric that the agent achieves on the ML problem it is been tested on, So it is not assessing the model reasoning and the choice of appropriate EDA methods according to the data. And it do not test the model understanding of the given data</t>
+  </si>
+  <si>
     <t xml:space="preserve">TemporalBench: A Benchmark for Evaluating LLM-Based Agents on Contextual and Event-Informed Time Series Tasks </t>
   </si>
   <si>
@@ -269,7 +252,9 @@
     <t xml:space="preserve">https://arxiv.org/abs/2602.13272</t>
   </si>
   <si>
-    <t xml:space="preserve">- It has time-series tasks in the evaluation.</t>
+    <t xml:space="preserve">'- Evaluates LLMs on distinct aspects of temporal reasoning.
+- It has 4 task families, forming an eval sequence that probes how temporal understanding and forecasting behavior change as additional sources of info are introduces.
+- tasks are: historical time-series understanding, and forecasting, both of which once without having a context and another after adding a context or prediction under specific future events.</t>
   </si>
   <si>
     <t xml:space="preserve">- 1) multiple-choice question answering tasks including (T1, T3), and the qualitative components of T2 and T4 :
@@ -285,6 +270,10 @@
     - OW_RMSSE</t>
   </si>
   <si>
+    <t xml:space="preserve">Paper focuses on time-series understanding and forecasting with context and without, comparing performance drop when adding it. Not measuring EDA performance.
+Paper shows that models with strong predictions are not necessarily has correct decisions when adding context or future condition events.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSRBENCH: A Comprehensive Multi-task Multi-modal Time Series Reasoning Benchmark for Generalist Models </t>
   </si>
   <si>
@@ -297,14 +286,55 @@
     <t xml:space="preserve">https://arxiv.org/abs/2601.18744</t>
   </si>
   <si>
-    <t xml:space="preserve">test multiple categories of LLMs, either VLMs, general LLMs, Time-series LLMs.
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">test multiple categories of LLMs, either VLMs, general LLMs, Time-series LLMs.
 And test on different modalities, either embedded, textual, visual or both.
 - It has questions including chaotic data, specifically “Lorenz Attractor”.
-It tests different aspects, like perception, reasoning decision and prediction. </t>
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">- 4125 problems from 14 domains, categorized into 4 aspects, testing: perception, reasoning decision making and prediction. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">“Accuracy” is mentioned to be the primary metric in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">experiments section.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Models still struggle with non-periodic, heterogeneous scientific signals. Which chaotic signals are the extreme case of this.
-Not focused on EDA or Data analysis.</t>
+Not focused on EDA or Data analysis.
+Used Eval. Metrics are not discussed sufficiently, and I think they are not representative to LLMs performance on each task.</t>
   </si>
   <si>
     <t xml:space="preserve">TSAQA: Time Series Analysis Question And Answering Benchmark </t>
@@ -353,7 +383,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -413,29 +443,18 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -501,7 +520,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -542,16 +561,8 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -856,16 +867,19 @@
       <c r="F4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="5" t="s">
         <v>28</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>29</v>
       </c>
+      <c r="I4" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="58.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>2024</v>
@@ -874,24 +888,27 @@
         <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="11" t="s">
         <v>32</v>
       </c>
+      <c r="E5" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="F5" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" s="11" t="s">
         <v>35</v>
       </c>
+      <c r="H5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="75.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>36</v>
+      <c r="A6" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>2026</v>
@@ -900,22 +917,25 @@
         <v>25</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="11" t="s">
-        <v>37</v>
+      <c r="E6" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="118" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>41</v>
+      <c r="A7" s="5" t="s">
+        <v>44</v>
       </c>
       <c r="B7" s="6" t="n">
         <v>2026</v>
@@ -923,26 +943,28 @@
       <c r="C7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>43</v>
+      <c r="D7" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>46</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="75.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>47</v>
+      <c r="A8" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="B8" s="6" t="n">
         <v>2026</v>
@@ -951,20 +973,20 @@
         <v>25</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="12" t="s">
-        <v>48</v>
+      <c r="E8" s="9" t="s">
+        <v>52</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>54</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>